<commit_message>
Fix sematic of number format and refactor number format saving
The predefined formats could have separate XLNumberFormatKey entries. E.g.,
format code '0.00' is a predefined number format 2 and it could be
be present in the structures under different numberFormatId (e.g. 164).

This is no longer possible, if format matches predefined format,
the numberFormatId is always correct one from the
XLPredefinedFormat.FormatCodes.

The consequence is that several test files had removed these extra entries
<numFmt numFmtId="164" formatCode="0.00" /> (or similar) the the various
places now reference correct predefined numFmtId instead of user added
number format id.
</commit_message>
<xml_diff>
--- a/ClosedXML.Tests/Resource/Examples/Misc/CellValues.xlsx
+++ b/ClosedXML.Tests/Resource/Examples/Misc/CellValues.xlsx
@@ -73,10 +73,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:numFmts count="3">
+  <x:numFmts count="2">
     <x:numFmt numFmtId="0" formatCode=""/>
     <x:numFmt numFmtId="164" formatCode="yyyy-MMM-dd"/>
-    <x:numFmt numFmtId="165" formatCode="#,##0.00"/>
   </x:numFmts>
   <x:fonts count="2">
     <x:font>
@@ -143,7 +142,7 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="4" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:protection locked="1" hidden="0"/>
     </x:xf>
     <x:xf numFmtId="46" fontId="0" fillId="0" borderId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
@@ -171,7 +170,7 @@
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>
-    <x:xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
+    <x:xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="0" applyAlignment="1" applyProtection="1">
       <x:alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" relativeIndent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
       <x:protection locked="1" hidden="0"/>
     </x:xf>

</xml_diff>